<commit_message>
Ageing: single CSV for all scenarios, canonical "Date" column
The CSV output was one file per scenario. Emit a single file instead,
tagging each row with a `scenario` column inserted right after `Date`,
so downstream consumers get every scenario in one place. Rows are
ordered by date, then by the workbook sheet order (Central first).

The Excel output is unchanged: still one sheet per scenario.

Scenario sheets are authored by hand and disagree on the date header
casing ("Date" vs "date"). Normalize it to the canonical `Date` at read
time so the ageing logic and both output headers stay stable regardless
of how a sheet is written.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/localRun/ageing/input/MAIWENN_EXP_INPUT_scn_ifrs9_25Q2_Def15may_secto_v9.xlsx
+++ b/localRun/ageing/input/MAIWENN_EXP_INPUT_scn_ifrs9_25Q2_Def15may_secto_v9.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mehdi\IdeaProjects\file_transform_engine\localRun\ageing\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF515E7-6762-4590-9473-EDD94CFF627D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B869588C-5D12-4D4F-B2CB-A19669125A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Central" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="24">
   <si>
     <t>IR_10Y_BE</t>
   </si>
@@ -40,9 +40,6 @@
     <t>CPI_YOY_US</t>
   </si>
   <si>
-    <t>CRE_PRICE_YOY*</t>
-  </si>
-  <si>
     <t>2025Q1</t>
   </si>
   <si>
@@ -92,6 +89,12 @@
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>CRE_PRICE_YOY</t>
   </si>
 </sst>
 </file>
@@ -481,12 +484,12 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" s="3">
         <v>3.1485469000000002E-2</v>
@@ -509,7 +512,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="3">
         <v>3.1167231E-2</v>
@@ -532,7 +535,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3">
         <v>3.2358333000000003E-2</v>
@@ -555,7 +558,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="3">
         <v>3.1785000000000001E-2</v>
@@ -578,7 +581,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="3">
         <v>3.0980000000000001E-2</v>
@@ -601,7 +604,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="3">
         <v>3.0980000000000001E-2</v>
@@ -624,7 +627,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3">
         <v>3.0980000000000001E-2</v>
@@ -647,7 +650,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" s="3">
         <v>3.0980000000000001E-2</v>
@@ -670,7 +673,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="3">
         <v>3.0980000000000001E-2</v>
@@ -693,7 +696,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="3">
         <v>3.0980000000000001E-2</v>
@@ -716,7 +719,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" s="3">
         <v>3.0980000000000001E-2</v>
@@ -739,7 +742,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" s="3">
         <v>3.0980000000000001E-2</v>
@@ -762,7 +765,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" s="3">
         <v>3.0980000000000001E-2</v>
@@ -785,7 +788,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15" s="3">
         <v>3.0980000000000001E-2</v>
@@ -808,7 +811,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" s="3">
         <v>3.0980000000000001E-2</v>
@@ -831,7 +834,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" s="3">
         <v>3.0980000000000001E-2</v>
@@ -863,12 +866,13 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="7" width="16" customWidth="1"/>
+    <col min="2" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="17.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -886,12 +890,12 @@
         <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" s="3">
         <v>3.1485470000000002E-2</v>
@@ -914,7 +918,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="3">
         <v>3.1167230000000001E-2</v>
@@ -937,7 +941,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3">
         <v>3.2358329999999998E-2</v>
@@ -960,7 +964,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="3">
         <v>3.1785000000000001E-2</v>
@@ -983,7 +987,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="3">
         <v>3.1230000000000001E-2</v>
@@ -1006,7 +1010,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="3">
         <v>3.073E-2</v>
@@ -1029,7 +1033,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3">
         <v>2.9229999999999999E-2</v>
@@ -1052,7 +1056,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" s="3">
         <v>2.7730000000000001E-2</v>
@@ -1075,7 +1079,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="3">
         <v>2.673E-2</v>
@@ -1098,7 +1102,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="3">
         <v>2.623E-2</v>
@@ -1121,7 +1125,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" s="3">
         <v>2.5729999999999999E-2</v>
@@ -1144,7 +1148,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" s="3">
         <v>2.4979999999999999E-2</v>
@@ -1167,7 +1171,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" s="3">
         <v>2.4729999999999999E-2</v>
@@ -1190,7 +1194,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15" s="3">
         <v>2.5229999999999999E-2</v>
@@ -1213,7 +1217,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" s="3">
         <v>2.5729999999999999E-2</v>
@@ -1236,7 +1240,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" s="3">
         <v>2.623E-2</v>
@@ -1268,12 +1272,13 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="7" width="16" customWidth="1"/>
+    <col min="2" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="17.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1291,12 +1296,12 @@
         <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" s="3">
         <v>3.1485470000000002E-2</v>
@@ -1319,7 +1324,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="3">
         <v>3.1167230000000001E-2</v>
@@ -1342,7 +1347,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3">
         <v>3.2358329999999998E-2</v>
@@ -1365,7 +1370,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="3">
         <v>3.1785000000000001E-2</v>
@@ -1388,7 +1393,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="3">
         <v>3.1230000000000001E-2</v>
@@ -1411,7 +1416,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="3">
         <v>3.1980000000000001E-2</v>
@@ -1434,7 +1439,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3">
         <v>3.2730000000000002E-2</v>
@@ -1457,7 +1462,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" s="3">
         <v>3.3480000000000003E-2</v>
@@ -1480,7 +1485,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="3">
         <v>3.4229999999999997E-2</v>
@@ -1503,7 +1508,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="3">
         <v>3.4729999999999997E-2</v>
@@ -1526,7 +1531,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" s="3">
         <v>3.5229999999999997E-2</v>
@@ -1549,7 +1554,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" s="3">
         <v>3.5729999999999998E-2</v>
@@ -1572,7 +1577,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" s="3">
         <v>3.5979999999999998E-2</v>
@@ -1595,7 +1600,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15" s="3">
         <v>3.5979999999999998E-2</v>
@@ -1618,7 +1623,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" s="3">
         <v>3.5979999999999998E-2</v>
@@ -1641,7 +1646,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" s="3">
         <v>3.5979999999999998E-2</v>
@@ -1678,7 +1683,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1696,12 +1701,12 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" s="3">
         <v>3.1485470000000002E-2</v>
@@ -1724,7 +1729,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="3">
         <v>3.1167230000000001E-2</v>
@@ -1747,7 +1752,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3">
         <v>3.2358329999999998E-2</v>
@@ -1770,7 +1775,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="3">
         <v>3.1785000000000001E-2</v>
@@ -1793,7 +1798,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="3">
         <v>3.2230000000000002E-2</v>
@@ -1816,7 +1821,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="3">
         <v>3.2730000000000002E-2</v>
@@ -1839,7 +1844,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3">
         <v>3.1230000000000001E-2</v>
@@ -1862,7 +1867,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" s="3">
         <v>2.9729999999999999E-2</v>
@@ -1885,7 +1890,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="3">
         <v>2.8729999999999999E-2</v>
@@ -1908,7 +1913,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="3">
         <v>2.8230000000000002E-2</v>
@@ -1931,7 +1936,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" s="3">
         <v>2.7730000000000001E-2</v>
@@ -1954,7 +1959,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" s="3">
         <v>2.673E-2</v>
@@ -1977,7 +1982,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" s="3">
         <v>2.5729999999999999E-2</v>
@@ -2000,7 +2005,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B15" s="3">
         <v>2.5229999999999999E-2</v>
@@ -2023,7 +2028,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" s="3">
         <v>2.4729999999999999E-2</v>
@@ -2046,7 +2051,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" s="3">
         <v>2.4230000000000002E-2</v>

</xml_diff>